<commit_message>
feat(gap-06): worker role with limited permissions + access tests
Custom Worker role (19 ACL keys: dashboard, catalog, sales orders/
invoices/shipments, customer listing, sales reports). No user
management, configuration, or deletes. Seeded worker@classy.local
and customer@classy.local. Pest 3/3: worker 200 on allowed pages,
401 on roles/users/configuration; admin still allowed.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -750,7 +750,11 @@
           <t>Use default customer auth; confirm password reset email works</t>
         </is>
       </c>
-      <c r="F5" s="19" t="n"/>
+      <c r="F5" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G5" s="14" t="inlineStr">
         <is>
           <t>Day 1</t>
@@ -905,7 +909,11 @@
           <t>Create a 'Worker' role in the admin ACL; restrict sensitive pages</t>
         </is>
       </c>
-      <c r="F10" s="19" t="n"/>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G10" s="14" t="inlineStr">
         <is>
           <t>Day 1</t>
@@ -1375,10 +1383,14 @@
       <c r="D6" s="19" t="n"/>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F6" s="19" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Worker role (custom, 19 keys) + worker@classy.local seeded; Pest 3/3 pass: worker 200 dashboard/products/orders, 401 roles/users/config</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="11">
       <c r="A7" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(gap-02,03,07): UGX fashion catalog, 16 products, 67 variants
UGX currency added as channel base. Demo products wiped (no orders).
10 configurables (size/colour) + 6 simples, fixed UGX prices, stock
per variant, placeholder images. Verified: category API, search,
product page with USh pricing.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -785,7 +785,11 @@
           <t>Use configurable products for size/colour variants</t>
         </is>
       </c>
-      <c r="F6" s="19" t="n"/>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G6" s="14" t="inlineStr">
         <is>
           <t>Day 1</t>
@@ -816,7 +820,11 @@
           <t>Use the product status toggle</t>
         </is>
       </c>
-      <c r="F7" s="19" t="n"/>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G7" s="14" t="inlineStr">
         <is>
           <t>Day 1</t>
@@ -847,7 +855,11 @@
           <t>Run a full test order on Day 1</t>
         </is>
       </c>
-      <c r="F8" s="19" t="n"/>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
           <t>Day 1</t>
@@ -944,7 +956,11 @@
           <t>Set inventory per variant</t>
         </is>
       </c>
-      <c r="F11" s="19" t="n"/>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G11" s="14" t="inlineStr">
         <is>
           <t>Day 1</t>
@@ -1435,10 +1451,14 @@
       <c r="D8" s="19" t="n"/>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F8" s="19" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>16 fashion products (10 configurable+6 simple, 67 variants) in UGX; category API + search verified; demo products wiped</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="11">
       <c r="A9" s="14" t="inlineStr">

</xml_diff>

<commit_message>
fix(plan): unverify cart/checkout until E2E order test passes
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -855,11 +855,7 @@
           <t>Run a full test order on Day 1</t>
         </is>
       </c>
-      <c r="F8" s="19" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+      <c r="F8" s="19" t="n"/>
       <c r="G8" s="14" t="inlineStr">
         <is>
           <t>Day 1</t>

</xml_diff>

<commit_message>
feat(gap-04): end-to-end configurable checkout test
Customer adds size/colour variant, checks out COD + flat rate,
pending UGX order created and visible in order history. 15 assertions.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -855,7 +855,11 @@
           <t>Run a full test order on Day 1</t>
         </is>
       </c>
-      <c r="F8" s="19" t="n"/>
+      <c r="F8" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G8" s="14" t="inlineStr">
         <is>
           <t>Day 1</t>
@@ -1204,7 +1208,11 @@
           <t>Theme tweaks</t>
         </is>
       </c>
-      <c r="F19" s="19" t="n"/>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Partly</t>
+        </is>
+      </c>
       <c r="G19" s="14" t="inlineStr">
         <is>
           <t>Day 1</t>
@@ -1423,10 +1431,14 @@
       <c r="D7" s="19" t="n"/>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F7" s="19" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>Name+logo+favicon live (header shows logo). Primary-colour token change + asset rebuild running</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="11">
       <c r="A8" s="14" t="inlineStr">
@@ -1475,10 +1487,14 @@
       <c r="D9" s="19" t="n"/>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F9" s="19" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Pest CheckoutFlowTest 15 assertions: variant cart, COD+flatrate, pending UGX order, history visible</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="11">
       <c r="A10" s="14" t="inlineStr">
@@ -1499,10 +1515,14 @@
       <c r="D10" s="19" t="n"/>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F10" s="19" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F10" s="19" t="inlineStr">
+        <is>
+          <t>Provider deferred by owner; Day 2 builds sandbox payment method (Flutterwave/Pesapal)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="11">
       <c r="A11" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(gap-15): brand theme plum + rebuild shop assets
navyBlue token redefined #060C3B -> #4A1942 to match Classy Fashion
Hub identity; shop assets rebuilt with npm. Logo/favicon/name live.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -1210,7 +1210,7 @@
       </c>
       <c r="F19" s="19" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G19" s="14" t="inlineStr">
@@ -1431,12 +1431,12 @@
       <c r="D7" s="19" t="n"/>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F7" s="19" t="inlineStr">
         <is>
-          <t>Name+logo+favicon live (header shows logo). Primary-colour token change + asset rebuild running</t>
+          <t>Name+logo+favicon live; navyBlue token redefined to plum #4A1942, shop assets rebuilt (rgb 74 25 66 in CSS)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(gap-09): report order statuses with guarded transitions
Pending>Confirmed>Paid>Processing>Dispatched>Delivered. ClassyFashion
package: transition map, manual status route (staff permission +
422 on illegal jumps), completed>dispatched auto-map on shipment,
admin buttons via view event, admin lang override. Core Order.php
gains 4 status codes/labels (no seam to extend); OrderStatusTest 5/5.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -1022,7 +1022,11 @@
           <t>Rename or extend default statuses; update status transitions</t>
         </is>
       </c>
-      <c r="F13" s="19" t="n"/>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G13" s="14" t="inlineStr">
         <is>
           <t>Day 2</t>
@@ -1543,10 +1547,14 @@
       <c r="D11" s="19" t="n"/>
       <c r="E11" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F11" s="19" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F11" s="19" t="inlineStr">
+        <is>
+          <t>Full pending&gt;confirmed&gt;paid&gt;processing&gt;dispatched&gt;delivered flow; OrderStatusTest 5/5 (19 assertions); completed auto-maps to dispatched</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="11">
       <c r="A12" s="14" t="inlineStr">
@@ -1567,10 +1575,14 @@
       <c r="D12" s="19" t="n"/>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F12" s="19" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Delivery fields: reading checkout address flow next</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="11">
       <c r="A13" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(gap-10): delivery instructions at checkout and admin view
addresses.delivery_instructions (migration, 500 chars). Shipping form
field via shop view event (vee-validate max:500); cart>order resource
chain extended (2 small core list additions, documented). Admin order
view shows instructions via address events. Tests: form renders,
persists to order, visible to admin.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -1057,7 +1057,11 @@
           <t>Add fields at checkout and show in admin order view</t>
         </is>
       </c>
-      <c r="F14" s="19" t="n"/>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G14" s="14" t="inlineStr">
         <is>
           <t>Day 2</t>
@@ -1575,12 +1579,12 @@
       <c r="D12" s="19" t="n"/>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F12" s="19" t="inlineStr">
         <is>
-          <t>Delivery fields: reading checkout address flow next</t>
+          <t>delivery_instructions on addresses table; shipping form field (Vue event), cart&gt;order flow, admin display; CheckoutFlowTest +2 assertions</t>
         </is>
       </c>
     </row>
@@ -1603,10 +1607,14 @@
       <c r="D13" s="19" t="n"/>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F13" s="19" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F13" s="19" t="inlineStr">
+        <is>
+          <t>Audit log: evaluating activity-log package next</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="11">
       <c r="A14" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(gap-12): audit trail for stock and order changes
Spatie activitylog v4 (PHP 8.3 compatible). Inventory observer logs
staff stock edits (old/new qty, source); status controller + auto-map
listener log manual/system transitions. AuditLogTest 4/4.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -1123,7 +1123,11 @@
           <t>Add a Laravel activity-log package recording user and date</t>
         </is>
       </c>
-      <c r="F16" s="19" t="n"/>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G16" s="14" t="inlineStr">
         <is>
           <t>Day 2</t>
@@ -1607,12 +1611,12 @@
       <c r="D13" s="19" t="n"/>
       <c r="E13" s="19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F13" s="19" t="inlineStr">
         <is>
-          <t>Audit log: evaluating activity-log package next</t>
+          <t>Spatie v4 activity log: stock observer + order audit; AuditLogTest 4/4 (16 assertions)</t>
         </is>
       </c>
     </row>
@@ -1635,10 +1639,14 @@
       <c r="D14" s="19" t="n"/>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F14" s="19" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F14" s="19" t="inlineStr">
+        <is>
+          <t>Low-stock: threshold + alert next</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="11">
       <c r="A15" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(gap-08): low-stock threshold and alerts
Threshold default 5 (seeded config). Existing dashboard widget
verified via stats API. Observer logs stock.low crossings with
qty/threshold. AuditLogTest 6/6.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -991,7 +991,11 @@
           <t>Add threshold field plus admin notice or email</t>
         </is>
       </c>
-      <c r="F12" s="19" t="n"/>
+      <c r="F12" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G12" s="14" t="inlineStr">
         <is>
           <t>Day 2</t>
@@ -1639,12 +1643,12 @@
       <c r="D14" s="19" t="n"/>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>Low-stock: threshold + alert next</t>
+          <t>Threshold=5 seeded; dashboard widget verified via stats API; crossings logged stock.low; AuditLogTest 6/6</t>
         </is>
       </c>
     </row>
@@ -1667,10 +1671,14 @@
       <c r="D15" s="19" t="n"/>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F15" s="19" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Cost price + profit next</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="11">
       <c r="A16" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(gap-13): cost price and profit per sale
Cost seeded at 60% of price. Profit helper (variant cost, parent
fallback); per-item + order profit on admin order view via events.
ProfitTest 3/3. Full suite 19/19.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -1162,7 +1162,11 @@
           <t>Add cost price to products; compute profit on order items</t>
         </is>
       </c>
-      <c r="F17" s="19" t="n"/>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G17" s="14" t="inlineStr">
         <is>
           <t>Day 2</t>
@@ -1671,12 +1675,12 @@
       <c r="D15" s="19" t="n"/>
       <c r="E15" s="19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>Cost price + profit next</t>
+          <t>Cost=60% price seeded; per-item + order profit on admin view; ProfitTest 3/3</t>
         </is>
       </c>
     </row>
@@ -1699,10 +1703,14 @@
       <c r="D16" s="19" t="n"/>
       <c r="E16" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F16" s="19" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F16" s="19" t="inlineStr">
+        <is>
+          <t>Mobile-money sandbox payment method (provider TBD)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="11">
       <c r="A17" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(gap-11): flutterwave mobile money in sandbox mode
Redirect-style MTN/Airtel method (UGX only, keys from .env).
Attempts table keeps pending/success/failed + tx refs. Order
created only after webhook signature + server-side verify
(amount/currency/tx_ref match); returns never create orders.
Status page doubles as verifier for localhost demo. Tests 6/6.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -1096,7 +1096,11 @@
           <t>Flutterwave or Pesapal payment method; mark Paid only after webhook confirmation; use sandbox</t>
         </is>
       </c>
-      <c r="F15" s="19" t="n"/>
+      <c r="F15" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G15" s="14" t="inlineStr">
         <is>
           <t>Day 2-3</t>
@@ -1703,12 +1707,12 @@
       <c r="D16" s="19" t="n"/>
       <c r="E16" s="19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>Mobile-money sandbox payment method (provider TBD)</t>
+          <t>Flutterwave UGX method (sandbox): pending attempts, signed webhook + verify create paid order; MobileMoneyTest 6/6. Live keys pending owner sandbox account</t>
         </is>
       </c>
     </row>
@@ -1731,10 +1735,14 @@
       <c r="D17" s="19" t="n"/>
       <c r="E17" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F17" s="19" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F17" s="19" t="inlineStr">
+        <is>
+          <t>Day-3: reports, phone test, docs</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="11">
       <c r="A18" s="14" t="inlineStr">

</xml_diff>

<commit_message>
feat(day3): sales reports verified, demo orders, robust tests
ReportingTest (stats + CSV export). DemoOrdersSeeder: 3 real UGX
orders (pending/paid/delivered) for screenshots. Tests hardened
against committed demo rows. Suite 27/27.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -890,7 +890,11 @@
           <t>Light customisation; check export options</t>
         </is>
       </c>
-      <c r="F9" s="19" t="n"/>
+      <c r="F9" s="19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="G9" s="14" t="inlineStr">
         <is>
           <t>Day 3</t>
@@ -1787,10 +1791,14 @@
       <c r="D19" s="19" t="n"/>
       <c r="E19" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F19" s="19" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F19" s="19" t="inlineStr">
+        <is>
+          <t>Sales stats + CSV export verified (ReportingTest); 3 demo orders; dashboard overall stats live</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="11">
       <c r="A20" s="14" t="inlineStr">

</xml_diff>

<commit_message>
docs(day3): user guide, demo script, limitations; plan finalized
USER_GUIDE (customer/worker/admin), DEMO_SCRIPT (6 SMART objectives
+ screenshot points), KNOWN_LIMITATIONS (sandbox, cuts, edges).
Notifications: admin notices verified; emails dashboard-only.
</commit_message>
<xml_diff>
--- a/Classy_Fashion_Hub_Bagisto_Plan.xlsx
+++ b/Classy_Fashion_Hub_Bagisto_Plan.xlsx
@@ -1062,12 +1062,12 @@
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Add fields at checkout and show in admin order view</t>
+          <t>Admin new-order notices verified (3 rows); customer order emails built-in but SMTP unconfigured -&gt; dashboard-only per cut order</t>
         </is>
       </c>
       <c r="F14" s="19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Partly</t>
         </is>
       </c>
       <c r="G14" s="14" t="inlineStr">
@@ -1167,12 +1167,12 @@
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Add cost price to products; compute profit on order items</t>
+          <t>Cut per plan (first cut). English only; noted as future work in KNOWN_LIMITATIONS.md</t>
         </is>
       </c>
       <c r="F17" s="19" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G17" s="14" t="inlineStr">
@@ -1543,12 +1543,12 @@
       <c r="D10" s="19" t="n"/>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="19" t="inlineStr">
         <is>
-          <t>Provider deferred by owner; Day 2 builds sandbox payment method (Flutterwave/Pesapal)</t>
+          <t>Flutterwave picked; method built+tested Day 2. Owner step: free sandbox account -&gt; test keys in bagisto/.env (README has steps)</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1739,12 @@
       <c r="D17" s="19" t="n"/>
       <c r="E17" s="19" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F17" s="19" t="inlineStr">
         <is>
-          <t>Day-3: reports, phone test, docs</t>
+          <t>MobileMoneyTest 6/6 (pending/verify/paid, bad signature, mismatch, return-proves-nothing). Live keys + public webhook URL still owner-side</t>
         </is>
       </c>
     </row>
@@ -1815,10 +1815,14 @@
       <c r="D20" s="19" t="n"/>
       <c r="E20" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F20" s="19" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F20" s="19" t="inlineStr">
+        <is>
+          <t>6/6 mapped in DEMO_SCRIPT; screenshots are owner-side (browser/phone)</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="11">
       <c r="A21" s="14" t="inlineStr">
@@ -1835,10 +1839,14 @@
       <c r="D21" s="19" t="n"/>
       <c r="E21" s="19" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F21" s="19" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F21" s="19" t="inlineStr">
+        <is>
+          <t>USER_GUIDE.md, DEMO_SCRIPT.md (6 objectives + shots), KNOWN_LIMITATIONS.md written</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E5:E21">

</xml_diff>